<commit_message>
docs(tracker): fix 3 stale Epic 1 sprint labels (100% but mislabeled)
Follow-up (6/6), Sprint 3 -- Plan gates + AI consent + 2FA (7/7), and Workflow as
Engine (16/16) were all fully done but still labeled In Progress/Backlog. Flipped to
Done. Epic 1 stays 94/105 (90%) In Progress -- the real remaining work is the S5
go-live/ops tier (observability, CI/CD, secrets manager, backups, load test) + S4-07
brain tool registry; none of those are secretly done.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic1_Stability.xlsx
+++ b/docs/DecisionOS_Epic1_Stability.xlsx
@@ -874,6 +874,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
@@ -964,7 +965,7 @@
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr"/>
@@ -1086,7 +1087,7 @@
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G11" s="10" t="inlineStr"/>
@@ -1173,7 +1174,7 @@
       </c>
       <c r="F14" s="12" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr"/>

</xml_diff>

<commit_message>
Epic 1 S4-07 DONE: central agent-tool registry in brain_router.py -> Sprint 4 17/17
brain.py compute handlers already used a central _COMPUTE_HANDLERS dict registry.
Formalized the 4 brain_router.py agent tools the same way: a _TOOL_HANDLERS registry
(name -> adapter) replaces the if/elif dispatch in _run_tools. Adding a tool = define
_tool_<name> + one registry line; the dispatcher never changes. Pydantic in/out wrapping
deliberately skipped -- these are internal handlers with consistent contracts, so
boundary-layer model ceremony adds no value here.

Verified: compile + ruff clean + route-fingerprint 266 unchanged. Sprint 4 -> 17/17 Done;
Epic 1 95/105 (90%, still In Progress -- the S5 go-live/ops tier remains). Master 401/605.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic1_Stability.xlsx
+++ b/docs/DecisionOS_Epic1_Stability.xlsx
@@ -870,7 +870,7 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Epic 1 progress: 94 of 105 items resolved  (90%)</t>
+          <t>Epic 1 progress: 95 of 105 items resolved  (90%)</t>
         </is>
       </c>
     </row>
@@ -1104,19 +1104,19 @@
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>17</v>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr"/>
@@ -4175,7 +4175,7 @@
       </c>
       <c r="J40" s="26" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K40" s="17" t="n"/>
@@ -4186,7 +4186,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O40" s="17" t="n"/>
+      <c r="O40" s="17" t="inlineStr">
+        <is>
+          <t>DONE 2026-08-27: brain.py compute handlers already used a central _COMPUTE_HANDLERS dict registry; formalized the 4 brain_router.py agent tools the same way (_TOOL_HANDLERS registry + adapter, replacing the if/elif dispatch). Add a tool = define _tool_&lt;name&gt; + one registry line. Pydantic in/out wrapping deliberately skipped -- these are internal handlers with consistent (ctx,plan,recs)/(t,user) contracts; Pydantic ceremony adds no value off the API boundary.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="32" customHeight="1">
       <c r="A41" s="17" t="inlineStr">

</xml_diff>